<commit_message>
Actualizacion de la logica de cursos equivalentes
</commit_message>
<xml_diff>
--- a/salida/excel/consumo_horas_educacion_secundaria.xlsx
+++ b/salida/excel/consumo_horas_educacion_secundaria.xlsx
@@ -489,24 +489,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="35" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,60 +529,70 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Laboratorio de Biología</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Laboratorio de Biología_Incremento</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Laboratorio de Computadoras</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Computadoras_Incremento</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Física</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Física_Incremento</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Química</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Química_Incremento</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Taller</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Taller_Incremento</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Virtual_Incremento</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Total_Incremento</t>
         </is>
@@ -617,21 +629,27 @@
         <v>0</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="O2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="P2" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="Q2" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -666,21 +684,27 @@
         <v>0</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M3" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P3" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="O3" s="5" t="n">
+      <c r="Q3" s="5" t="n">
         <v>29</v>
       </c>
     </row>
@@ -691,16 +715,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0</v>
@@ -709,28 +733,34 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="O4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="N4" s="3" t="n">
-        <v>63</v>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>24</v>
+      <c r="P4" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -740,13 +770,13 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>23</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0</v>
@@ -758,27 +788,33 @@
         <v>0</v>
       </c>
       <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="O5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="I5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="M5" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="N5" s="5" t="n">
-        <v>93</v>
-      </c>
-      <c r="O5" s="5" t="n">
+      <c r="P5" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q5" s="5" t="n">
         <v>30</v>
       </c>
     </row>
@@ -789,13 +825,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>18</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0</v>
@@ -807,27 +843,33 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>113</v>
+        <v>13</v>
       </c>
       <c r="O6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q6" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -838,28 +880,28 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>32</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>3</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>4</v>
@@ -868,15 +910,21 @@
         <v>0</v>
       </c>
       <c r="L7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="M7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" s="5" t="n">
-        <v>159</v>
-      </c>
       <c r="O7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>161</v>
+      </c>
+      <c r="Q7" s="5" t="n">
         <v>46</v>
       </c>
     </row>
@@ -887,28 +935,28 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>26</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="G8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>10</v>
-      </c>
       <c r="I8" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>4</v>
@@ -917,15 +965,21 @@
         <v>0</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>188</v>
+        <v>16</v>
       </c>
       <c r="O8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q8" s="3" t="n">
         <v>29</v>
       </c>
     </row>
@@ -936,46 +990,52 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="K9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L9" s="5" t="n">
+      <c r="M9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="M9" s="5" t="n">
+      <c r="O9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="5" t="n">
-        <v>207</v>
-      </c>
-      <c r="O9" s="5" t="n">
-        <v>19</v>
+      <c r="P9" s="5" t="n">
+        <v>214</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -985,45 +1045,51 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="M10" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="N10" s="3" t="n">
-        <v>223</v>
-      </c>
       <c r="O10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="Q10" s="3" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1034,45 +1100,51 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>8</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="M11" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="N11" s="5" t="n">
-        <v>235</v>
-      </c>
       <c r="O11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="P11" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q11" s="5" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1083,47 +1155,53 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O12" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P12" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1132,47 +1210,53 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O13" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="P13" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1181,47 +1265,53 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O14" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P14" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1230,47 +1320,53 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O15" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="P15" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1279,47 +1375,53 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O16" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P16" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1328,47 +1430,53 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O17" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="P17" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1377,47 +1485,53 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O18" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P18" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q18" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1426,47 +1540,53 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O19" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="P19" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1475,47 +1595,53 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O20" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P20" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q20" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1524,45 +1650,51 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="M21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="O21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1577,7 +1709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1783,7 +1915,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -3411,7 +3543,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -3812,13 +3944,13 @@
         <v>3</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H60" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -3842,20 +3974,20 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F61" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G61" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H61" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I61" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
@@ -4397,7 +4529,7 @@
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F76" s="3" t="n">
@@ -4952,7 +5084,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F91" s="5" t="n">
@@ -5097,7 +5229,7 @@
       <c r="G95" s="8" t="inlineStr"/>
       <c r="H95" s="8" t="inlineStr"/>
       <c r="I95" s="8" t="n">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="96">
@@ -5152,7 +5284,7 @@
       <c r="C98" s="8" t="inlineStr"/>
       <c r="D98" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr"/>
@@ -5160,7 +5292,7 @@
       <c r="G98" s="8" t="inlineStr"/>
       <c r="H98" s="8" t="inlineStr"/>
       <c r="I98" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99">
@@ -5173,7 +5305,7 @@
       <c r="C99" s="8" t="inlineStr"/>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr"/>
@@ -5181,7 +5313,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100">
@@ -5194,7 +5326,7 @@
       <c r="C100" s="8" t="inlineStr"/>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr"/>
@@ -5202,24 +5334,45 @@
       <c r="G100" s="8" t="inlineStr"/>
       <c r="H100" s="8" t="inlineStr"/>
       <c r="I100" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr"/>
       <c r="C101" s="8" t="inlineStr"/>
-      <c r="D101" s="8" t="inlineStr"/>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E101" s="8" t="inlineStr"/>
       <c r="F101" s="8" t="inlineStr"/>
       <c r="G101" s="8" t="inlineStr"/>
       <c r="H101" s="8" t="inlineStr"/>
       <c r="I101" s="8" t="n">
-        <v>223</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B102" s="7" t="inlineStr"/>
+      <c r="C102" s="8" t="inlineStr"/>
+      <c r="D102" s="8" t="inlineStr"/>
+      <c r="E102" s="8" t="inlineStr"/>
+      <c r="F102" s="8" t="inlineStr"/>
+      <c r="G102" s="8" t="inlineStr"/>
+      <c r="H102" s="8" t="inlineStr"/>
+      <c r="I102" s="8" t="n">
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -5233,7 +5386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5439,7 +5592,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -7067,7 +7220,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -7579,13 +7732,13 @@
         <v>2</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -7609,20 +7762,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -8164,7 +8317,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -8719,7 +8872,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -8901,7 +9054,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -8956,7 +9109,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -8964,7 +9117,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -8977,7 +9130,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -8985,7 +9138,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -8998,7 +9151,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -9006,24 +9159,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -9037,7 +9211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9243,7 +9417,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -10871,7 +11045,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -11383,13 +11557,13 @@
         <v>5</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -11413,20 +11587,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>5</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -11968,7 +12142,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -12523,7 +12697,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -12705,7 +12879,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -12760,7 +12934,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -12768,7 +12942,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -12781,7 +12955,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -12789,7 +12963,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -12802,7 +12976,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -12810,24 +12984,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -12841,7 +13036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13047,7 +13242,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -14675,7 +14870,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -15187,13 +15382,13 @@
         <v>3</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -15217,20 +15412,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -15772,7 +15967,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -16327,7 +16522,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -16509,7 +16704,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -16564,7 +16759,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -16572,7 +16767,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -16585,7 +16780,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -16593,7 +16788,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -16606,7 +16801,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -16614,24 +16809,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -16645,7 +16861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16851,7 +17067,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -18479,7 +18695,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -18991,13 +19207,13 @@
         <v>4</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -19021,20 +19237,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>4</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -19576,7 +19792,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -20131,7 +20347,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -20313,7 +20529,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -20368,7 +20584,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -20376,7 +20592,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -20389,7 +20605,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -20397,7 +20613,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -20410,7 +20626,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -20418,24 +20634,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -20449,7 +20686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20655,7 +20892,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -22283,7 +22520,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -22795,13 +23032,13 @@
         <v>3</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -22825,20 +23062,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -23380,7 +23617,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -23935,7 +24172,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -24117,7 +24354,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -24172,7 +24409,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -24180,7 +24417,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -24193,7 +24430,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -24201,7 +24438,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -24214,7 +24451,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -24222,24 +24459,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -24253,7 +24511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -24459,7 +24717,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -26087,7 +26345,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -26599,13 +26857,13 @@
         <v>7</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -26629,20 +26887,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>7</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -27184,7 +27442,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -27739,7 +27997,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -27921,7 +28179,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -27976,7 +28234,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -27984,7 +28242,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -27997,7 +28255,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -28005,7 +28263,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -28018,7 +28276,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -28026,24 +28284,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -28057,7 +28336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28263,7 +28542,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -29891,7 +30170,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -30403,13 +30682,13 @@
         <v>3</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -30433,20 +30712,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -30988,7 +31267,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -31543,7 +31822,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -31725,7 +32004,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -31780,7 +32059,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -31788,7 +32067,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -31801,7 +32080,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -31809,7 +32088,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -31822,7 +32101,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -31830,24 +32109,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -31861,7 +32161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -32067,7 +32367,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -33695,7 +33995,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -34207,13 +34507,13 @@
         <v>7</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -34237,20 +34537,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>7</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -34792,7 +35092,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -35347,7 +35647,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -35529,7 +35829,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -35584,7 +35884,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -35592,7 +35892,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -35605,7 +35905,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -35613,7 +35913,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -35626,7 +35926,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -35634,24 +35934,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -35665,7 +35986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35871,7 +36192,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -37499,7 +37820,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -38011,13 +38332,13 @@
         <v>3</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -38041,20 +38362,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -38596,7 +38917,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -39151,7 +39472,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -39333,7 +39654,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -39388,7 +39709,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -39396,7 +39717,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -39409,7 +39730,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -39417,7 +39738,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -39430,7 +39751,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -39438,24 +39759,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -39748,7 +40090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -39954,7 +40296,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -41582,7 +41924,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -42094,13 +42436,13 @@
         <v>8</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -42124,20 +42466,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>8</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -42679,7 +43021,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -43234,7 +43576,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -43416,7 +43758,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -43471,7 +43813,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -43479,7 +43821,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -43492,7 +43834,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -43500,7 +43842,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -43513,7 +43855,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -43521,24 +43863,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -43552,7 +43915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -43758,7 +44121,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -45386,7 +45749,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -45898,13 +46261,13 @@
         <v>5</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -45928,20 +46291,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>5</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -46483,7 +46846,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -47038,7 +47401,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -47220,7 +47583,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100">
@@ -47275,7 +47638,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -47283,7 +47646,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -47296,7 +47659,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -47304,7 +47667,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -47317,7 +47680,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -47325,24 +47688,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -48107,7 +48491,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -48306,7 +48690,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -49040,13 +49424,13 @@
         <v>3</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H25" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -49070,20 +49454,20 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -49178,7 +49562,7 @@
       <c r="G29" s="8" t="inlineStr"/>
       <c r="H29" s="8" t="inlineStr"/>
       <c r="I29" s="8" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30">
@@ -49233,7 +49617,7 @@
       <c r="C32" s="8" t="inlineStr"/>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr"/>
@@ -49241,7 +49625,7 @@
       <c r="G32" s="8" t="inlineStr"/>
       <c r="H32" s="8" t="inlineStr"/>
       <c r="I32" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -49258,7 +49642,7 @@
       <c r="G33" s="8" t="inlineStr"/>
       <c r="H33" s="8" t="inlineStr"/>
       <c r="I33" s="8" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -49272,14 +49656,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -49478,7 +49862,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -50471,13 +50855,13 @@
         <v>1</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H32" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -50501,20 +50885,20 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F33" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H33" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
@@ -50831,7 +51215,7 @@
       <c r="G42" s="8" t="inlineStr"/>
       <c r="H42" s="8" t="inlineStr"/>
       <c r="I42" s="8" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43">
@@ -50886,7 +51270,7 @@
       <c r="C45" s="8" t="inlineStr"/>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr"/>
@@ -50894,24 +51278,45 @@
       <c r="G45" s="8" t="inlineStr"/>
       <c r="H45" s="8" t="inlineStr"/>
       <c r="I45" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr"/>
       <c r="C46" s="8" t="inlineStr"/>
-      <c r="D46" s="8" t="inlineStr"/>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Química</t>
+        </is>
+      </c>
       <c r="E46" s="8" t="inlineStr"/>
       <c r="F46" s="8" t="inlineStr"/>
       <c r="G46" s="8" t="inlineStr"/>
       <c r="H46" s="8" t="inlineStr"/>
       <c r="I46" s="8" t="n">
-        <v>93</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr"/>
+      <c r="C47" s="8" t="inlineStr"/>
+      <c r="D47" s="8" t="inlineStr"/>
+      <c r="E47" s="8" t="inlineStr"/>
+      <c r="F47" s="8" t="inlineStr"/>
+      <c r="G47" s="8" t="inlineStr"/>
+      <c r="H47" s="8" t="inlineStr"/>
+      <c r="I47" s="8" t="n">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -50925,14 +51330,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -51131,7 +51536,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -52198,13 +52603,13 @@
         <v>3</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H34" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -52228,20 +52633,20 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F35" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H35" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
@@ -52743,7 +53148,7 @@
       <c r="G49" s="8" t="inlineStr"/>
       <c r="H49" s="8" t="inlineStr"/>
       <c r="I49" s="8" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="50">
@@ -52798,7 +53203,7 @@
       <c r="C52" s="8" t="inlineStr"/>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr"/>
@@ -52806,24 +53211,45 @@
       <c r="G52" s="8" t="inlineStr"/>
       <c r="H52" s="8" t="inlineStr"/>
       <c r="I52" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr"/>
       <c r="C53" s="8" t="inlineStr"/>
-      <c r="D53" s="8" t="inlineStr"/>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Química</t>
+        </is>
+      </c>
       <c r="E53" s="8" t="inlineStr"/>
       <c r="F53" s="8" t="inlineStr"/>
       <c r="G53" s="8" t="inlineStr"/>
       <c r="H53" s="8" t="inlineStr"/>
       <c r="I53" s="8" t="n">
-        <v>113</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr"/>
+      <c r="C54" s="8" t="inlineStr"/>
+      <c r="D54" s="8" t="inlineStr"/>
+      <c r="E54" s="8" t="inlineStr"/>
+      <c r="F54" s="8" t="inlineStr"/>
+      <c r="G54" s="8" t="inlineStr"/>
+      <c r="H54" s="8" t="inlineStr"/>
+      <c r="I54" s="8" t="n">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -52837,7 +53263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -53043,7 +53469,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -54443,13 +54869,13 @@
         <v>2</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H43" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I43" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -54473,20 +54899,20 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H44" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
@@ -55028,7 +55454,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F59" s="5" t="n">
@@ -55358,7 +55784,7 @@
       <c r="G68" s="8" t="inlineStr"/>
       <c r="H68" s="8" t="inlineStr"/>
       <c r="I68" s="8" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69">
@@ -55413,7 +55839,7 @@
       <c r="C71" s="8" t="inlineStr"/>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr"/>
@@ -55421,7 +55847,7 @@
       <c r="G71" s="8" t="inlineStr"/>
       <c r="H71" s="8" t="inlineStr"/>
       <c r="I71" s="8" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72">
@@ -55434,7 +55860,7 @@
       <c r="C72" s="8" t="inlineStr"/>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr"/>
@@ -55442,7 +55868,7 @@
       <c r="G72" s="8" t="inlineStr"/>
       <c r="H72" s="8" t="inlineStr"/>
       <c r="I72" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
@@ -55455,7 +55881,7 @@
       <c r="C73" s="8" t="inlineStr"/>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr"/>
@@ -55463,24 +55889,45 @@
       <c r="G73" s="8" t="inlineStr"/>
       <c r="H73" s="8" t="inlineStr"/>
       <c r="I73" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr"/>
       <c r="C74" s="8" t="inlineStr"/>
-      <c r="D74" s="8" t="inlineStr"/>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E74" s="8" t="inlineStr"/>
       <c r="F74" s="8" t="inlineStr"/>
       <c r="G74" s="8" t="inlineStr"/>
       <c r="H74" s="8" t="inlineStr"/>
       <c r="I74" s="8" t="n">
-        <v>159</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr"/>
+      <c r="C75" s="8" t="inlineStr"/>
+      <c r="D75" s="8" t="inlineStr"/>
+      <c r="E75" s="8" t="inlineStr"/>
+      <c r="F75" s="8" t="inlineStr"/>
+      <c r="G75" s="8" t="inlineStr"/>
+      <c r="H75" s="8" t="inlineStr"/>
+      <c r="I75" s="8" t="n">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -55494,7 +55941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -55700,7 +56147,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -57359,13 +57806,13 @@
         <v>3</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H50" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -57389,20 +57836,20 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F51" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H51" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I51" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -57944,7 +58391,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F66" s="3" t="n">
@@ -58459,7 +58906,7 @@
       <c r="G80" s="8" t="inlineStr"/>
       <c r="H80" s="8" t="inlineStr"/>
       <c r="I80" s="8" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="81">
@@ -58514,7 +58961,7 @@
       <c r="C83" s="8" t="inlineStr"/>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr"/>
@@ -58522,7 +58969,7 @@
       <c r="G83" s="8" t="inlineStr"/>
       <c r="H83" s="8" t="inlineStr"/>
       <c r="I83" s="8" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="84">
@@ -58535,7 +58982,7 @@
       <c r="C84" s="8" t="inlineStr"/>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr"/>
@@ -58543,7 +58990,7 @@
       <c r="G84" s="8" t="inlineStr"/>
       <c r="H84" s="8" t="inlineStr"/>
       <c r="I84" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85">
@@ -58556,7 +59003,7 @@
       <c r="C85" s="8" t="inlineStr"/>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr"/>
@@ -58564,24 +59011,45 @@
       <c r="G85" s="8" t="inlineStr"/>
       <c r="H85" s="8" t="inlineStr"/>
       <c r="I85" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr"/>
       <c r="C86" s="8" t="inlineStr"/>
-      <c r="D86" s="8" t="inlineStr"/>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E86" s="8" t="inlineStr"/>
       <c r="F86" s="8" t="inlineStr"/>
       <c r="G86" s="8" t="inlineStr"/>
       <c r="H86" s="8" t="inlineStr"/>
       <c r="I86" s="8" t="n">
-        <v>188</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr"/>
+      <c r="C87" s="8" t="inlineStr"/>
+      <c r="D87" s="8" t="inlineStr"/>
+      <c r="E87" s="8" t="inlineStr"/>
+      <c r="F87" s="8" t="inlineStr"/>
+      <c r="G87" s="8" t="inlineStr"/>
+      <c r="H87" s="8" t="inlineStr"/>
+      <c r="I87" s="8" t="n">
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -58595,7 +59063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -58801,7 +59269,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -60429,7 +60897,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -60719,13 +61187,13 @@
         <v>2</v>
       </c>
       <c r="G57" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H57" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I57" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -60749,20 +61217,20 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F58" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H58" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -61304,7 +61772,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F73" s="5" t="n">
@@ -61859,7 +62327,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F88" s="3" t="n">
@@ -61893,7 +62361,7 @@
       <c r="G89" s="8" t="inlineStr"/>
       <c r="H89" s="8" t="inlineStr"/>
       <c r="I89" s="8" t="n">
-        <v>159</v>
+        <v>165</v>
       </c>
     </row>
     <row r="90">
@@ -61948,7 +62416,7 @@
       <c r="C92" s="8" t="inlineStr"/>
       <c r="D92" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr"/>
@@ -61956,7 +62424,7 @@
       <c r="G92" s="8" t="inlineStr"/>
       <c r="H92" s="8" t="inlineStr"/>
       <c r="I92" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93">
@@ -61969,7 +62437,7 @@
       <c r="C93" s="8" t="inlineStr"/>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr"/>
@@ -61977,7 +62445,7 @@
       <c r="G93" s="8" t="inlineStr"/>
       <c r="H93" s="8" t="inlineStr"/>
       <c r="I93" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">
@@ -61990,7 +62458,7 @@
       <c r="C94" s="8" t="inlineStr"/>
       <c r="D94" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr"/>
@@ -61998,24 +62466,45 @@
       <c r="G94" s="8" t="inlineStr"/>
       <c r="H94" s="8" t="inlineStr"/>
       <c r="I94" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr"/>
       <c r="C95" s="8" t="inlineStr"/>
-      <c r="D95" s="8" t="inlineStr"/>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E95" s="8" t="inlineStr"/>
       <c r="F95" s="8" t="inlineStr"/>
       <c r="G95" s="8" t="inlineStr"/>
       <c r="H95" s="8" t="inlineStr"/>
       <c r="I95" s="8" t="n">
-        <v>207</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr"/>
+      <c r="C96" s="8" t="inlineStr"/>
+      <c r="D96" s="8" t="inlineStr"/>
+      <c r="E96" s="8" t="inlineStr"/>
+      <c r="F96" s="8" t="inlineStr"/>
+      <c r="G96" s="8" t="inlineStr"/>
+      <c r="H96" s="8" t="inlineStr"/>
+      <c r="I96" s="8" t="n">
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion de Modalidad de Cursos
</commit_message>
<xml_diff>
--- a/salida/excel/consumo_horas_educacion_secundaria.xlsx
+++ b/salida/excel/consumo_horas_educacion_secundaria.xlsx
@@ -489,24 +489,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="35" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,60 +529,70 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Laboratorio de Biología</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Laboratorio de Biología_Incremento</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Laboratorio de Computadoras</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Computadoras_Incremento</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Física</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Física_Incremento</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Química</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Laboratorio de Química_Incremento</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Taller</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Taller_Incremento</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Virtual</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Virtual_Incremento</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Total_Incremento</t>
         </is>
@@ -617,21 +629,27 @@
         <v>0</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="O2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="P2" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="Q2" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -666,21 +684,27 @@
         <v>0</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M3" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P3" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="O3" s="5" t="n">
+      <c r="Q3" s="5" t="n">
         <v>29</v>
       </c>
     </row>
@@ -691,16 +715,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0</v>
@@ -709,28 +733,34 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="O4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="N4" s="3" t="n">
-        <v>63</v>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>24</v>
+      <c r="P4" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -740,13 +770,13 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>23</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0</v>
@@ -758,27 +788,33 @@
         <v>0</v>
       </c>
       <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="O5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="I5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="M5" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="N5" s="5" t="n">
-        <v>93</v>
-      </c>
-      <c r="O5" s="5" t="n">
+      <c r="P5" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q5" s="5" t="n">
         <v>30</v>
       </c>
     </row>
@@ -789,13 +825,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>18</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0</v>
@@ -807,27 +843,33 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>113</v>
+        <v>13</v>
       </c>
       <c r="O6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q6" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -838,28 +880,28 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>32</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>3</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>4</v>
@@ -868,15 +910,21 @@
         <v>0</v>
       </c>
       <c r="L7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="M7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" s="5" t="n">
-        <v>159</v>
-      </c>
       <c r="O7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>161</v>
+      </c>
+      <c r="Q7" s="5" t="n">
         <v>46</v>
       </c>
     </row>
@@ -887,28 +935,28 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>26</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="G8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>10</v>
-      </c>
       <c r="I8" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>4</v>
@@ -917,15 +965,21 @@
         <v>0</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>188</v>
+        <v>16</v>
       </c>
       <c r="O8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q8" s="3" t="n">
         <v>29</v>
       </c>
     </row>
@@ -936,46 +990,52 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="K9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L9" s="5" t="n">
+      <c r="M9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="M9" s="5" t="n">
+      <c r="O9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="5" t="n">
-        <v>207</v>
-      </c>
-      <c r="O9" s="5" t="n">
-        <v>19</v>
+      <c r="P9" s="5" t="n">
+        <v>214</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -985,45 +1045,51 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>16</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>223</v>
+        <v>16</v>
       </c>
       <c r="O10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="Q10" s="3" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1034,45 +1100,51 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>8</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="M11" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="N11" s="5" t="n">
-        <v>235</v>
-      </c>
       <c r="O11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="P11" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q11" s="5" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1083,47 +1155,53 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O12" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P12" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1132,47 +1210,53 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O13" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="P13" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1181,47 +1265,53 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O14" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P14" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1230,47 +1320,53 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O15" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="P15" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1279,47 +1375,53 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O16" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P16" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1328,47 +1430,53 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O17" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="P17" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1377,47 +1485,53 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O18" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P18" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q18" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1426,47 +1540,53 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O19" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="P19" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1475,47 +1595,53 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O20" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P20" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q20" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1524,45 +1650,51 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>235</v>
+        <v>20</v>
       </c>
       <c r="O21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="Q21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1577,7 +1709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1783,7 +1915,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -3411,7 +3543,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -3812,13 +3944,13 @@
         <v>3</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H60" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -3842,20 +3974,20 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F61" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G61" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H61" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I61" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
@@ -4397,7 +4529,7 @@
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F76" s="3" t="n">
@@ -4952,7 +5084,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F91" s="5" t="n">
@@ -5097,7 +5229,7 @@
       <c r="G95" s="8" t="inlineStr"/>
       <c r="H95" s="8" t="inlineStr"/>
       <c r="I95" s="8" t="n">
-        <v>175</v>
+        <v>181</v>
       </c>
     </row>
     <row r="96">
@@ -5152,7 +5284,7 @@
       <c r="C98" s="8" t="inlineStr"/>
       <c r="D98" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr"/>
@@ -5160,7 +5292,7 @@
       <c r="G98" s="8" t="inlineStr"/>
       <c r="H98" s="8" t="inlineStr"/>
       <c r="I98" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99">
@@ -5173,7 +5305,7 @@
       <c r="C99" s="8" t="inlineStr"/>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr"/>
@@ -5181,7 +5313,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100">
@@ -5194,7 +5326,7 @@
       <c r="C100" s="8" t="inlineStr"/>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr"/>
@@ -5202,24 +5334,45 @@
       <c r="G100" s="8" t="inlineStr"/>
       <c r="H100" s="8" t="inlineStr"/>
       <c r="I100" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr"/>
       <c r="C101" s="8" t="inlineStr"/>
-      <c r="D101" s="8" t="inlineStr"/>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E101" s="8" t="inlineStr"/>
       <c r="F101" s="8" t="inlineStr"/>
       <c r="G101" s="8" t="inlineStr"/>
       <c r="H101" s="8" t="inlineStr"/>
       <c r="I101" s="8" t="n">
-        <v>223</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B102" s="7" t="inlineStr"/>
+      <c r="C102" s="8" t="inlineStr"/>
+      <c r="D102" s="8" t="inlineStr"/>
+      <c r="E102" s="8" t="inlineStr"/>
+      <c r="F102" s="8" t="inlineStr"/>
+      <c r="G102" s="8" t="inlineStr"/>
+      <c r="H102" s="8" t="inlineStr"/>
+      <c r="I102" s="8" t="n">
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -5233,7 +5386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5439,7 +5592,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -7067,7 +7220,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -7579,13 +7732,13 @@
         <v>2</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -7609,20 +7762,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -8164,7 +8317,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -8719,7 +8872,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -8901,7 +9054,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -8956,7 +9109,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -8964,7 +9117,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -8977,7 +9130,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -8985,7 +9138,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -8998,7 +9151,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -9006,24 +9159,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -9037,7 +9211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9243,7 +9417,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -10871,7 +11045,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -11383,13 +11557,13 @@
         <v>5</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -11413,20 +11587,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>5</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -11968,7 +12142,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -12523,7 +12697,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -12705,7 +12879,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -12760,7 +12934,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -12768,7 +12942,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -12781,7 +12955,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -12789,7 +12963,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -12802,7 +12976,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -12810,24 +12984,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -12841,7 +13036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13047,7 +13242,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -14675,7 +14870,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -15187,13 +15382,13 @@
         <v>3</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -15217,20 +15412,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -15772,7 +15967,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -16327,7 +16522,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -16509,7 +16704,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -16564,7 +16759,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -16572,7 +16767,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -16585,7 +16780,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -16593,7 +16788,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -16606,7 +16801,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -16614,24 +16809,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -16645,7 +16861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16851,7 +17067,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -18479,7 +18695,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -18991,13 +19207,13 @@
         <v>4</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -19021,20 +19237,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>4</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -19576,7 +19792,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -20131,7 +20347,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -20313,7 +20529,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -20368,7 +20584,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -20376,7 +20592,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -20389,7 +20605,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -20397,7 +20613,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -20410,7 +20626,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -20418,24 +20634,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -20449,7 +20686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20655,7 +20892,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -22283,7 +22520,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -22795,13 +23032,13 @@
         <v>3</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -22825,20 +23062,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -23380,7 +23617,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -23935,7 +24172,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -24117,7 +24354,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -24172,7 +24409,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -24180,7 +24417,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -24193,7 +24430,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -24201,7 +24438,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -24214,7 +24451,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -24222,24 +24459,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -24253,7 +24511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -24459,7 +24717,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -26087,7 +26345,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -26599,13 +26857,13 @@
         <v>7</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -26629,20 +26887,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>7</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -27184,7 +27442,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -27739,7 +27997,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -27921,7 +28179,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -27976,7 +28234,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -27984,7 +28242,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -27997,7 +28255,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -28005,7 +28263,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -28018,7 +28276,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -28026,24 +28284,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -28057,7 +28336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28263,7 +28542,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -29891,7 +30170,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -30403,13 +30682,13 @@
         <v>3</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -30433,20 +30712,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -30988,7 +31267,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -31543,7 +31822,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -31725,7 +32004,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -31780,7 +32059,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -31788,7 +32067,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -31801,7 +32080,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -31809,7 +32088,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -31822,7 +32101,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -31830,24 +32109,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -31861,7 +32161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -32067,7 +32367,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -33695,7 +33995,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -34207,13 +34507,13 @@
         <v>7</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -34237,20 +34537,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>7</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -34792,7 +35092,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -35347,7 +35647,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -35529,7 +35829,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -35584,7 +35884,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -35592,7 +35892,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -35605,7 +35905,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -35613,7 +35913,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -35626,7 +35926,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -35634,24 +35934,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -35665,7 +35986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35871,7 +36192,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -37499,7 +37820,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -38011,13 +38332,13 @@
         <v>3</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -38041,20 +38362,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -38596,7 +38917,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -39151,7 +39472,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -39333,7 +39654,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -39388,7 +39709,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -39396,7 +39717,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -39409,7 +39730,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -39417,7 +39738,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -39430,7 +39751,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -39438,24 +39759,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -39748,7 +40090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -39954,7 +40296,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -41582,7 +41924,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -42094,13 +42436,13 @@
         <v>8</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -42124,20 +42466,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>8</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -42679,7 +43021,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -43234,7 +43576,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -43416,7 +43758,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -43471,7 +43813,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -43479,7 +43821,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -43492,7 +43834,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -43500,7 +43842,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -43513,7 +43855,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -43521,24 +43863,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -43552,7 +43915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -43758,7 +44121,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -45386,7 +45749,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -45898,13 +46261,13 @@
         <v>5</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -45928,20 +46291,20 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
         <v>5</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -46483,7 +46846,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F79" s="5" t="n">
@@ -47038,7 +47401,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F94" s="3" t="n">
@@ -47220,7 +47583,7 @@
       <c r="G99" s="8" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100">
@@ -47275,7 +47638,7 @@
       <c r="C102" s="8" t="inlineStr"/>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr"/>
@@ -47283,7 +47646,7 @@
       <c r="G102" s="8" t="inlineStr"/>
       <c r="H102" s="8" t="inlineStr"/>
       <c r="I102" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -47296,7 +47659,7 @@
       <c r="C103" s="8" t="inlineStr"/>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr"/>
@@ -47304,7 +47667,7 @@
       <c r="G103" s="8" t="inlineStr"/>
       <c r="H103" s="8" t="inlineStr"/>
       <c r="I103" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">
@@ -47317,7 +47680,7 @@
       <c r="C104" s="8" t="inlineStr"/>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr"/>
@@ -47325,24 +47688,45 @@
       <c r="G104" s="8" t="inlineStr"/>
       <c r="H104" s="8" t="inlineStr"/>
       <c r="I104" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr"/>
       <c r="C105" s="8" t="inlineStr"/>
-      <c r="D105" s="8" t="inlineStr"/>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E105" s="8" t="inlineStr"/>
       <c r="F105" s="8" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr"/>
       <c r="H105" s="8" t="inlineStr"/>
       <c r="I105" s="8" t="n">
-        <v>235</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr"/>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr"/>
+      <c r="F106" s="8" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr"/>
+      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="n">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -48107,7 +48491,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -48306,7 +48690,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -49040,13 +49424,13 @@
         <v>3</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H25" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -49070,20 +49454,20 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -49178,7 +49562,7 @@
       <c r="G29" s="8" t="inlineStr"/>
       <c r="H29" s="8" t="inlineStr"/>
       <c r="I29" s="8" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30">
@@ -49233,7 +49617,7 @@
       <c r="C32" s="8" t="inlineStr"/>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr"/>
@@ -49241,7 +49625,7 @@
       <c r="G32" s="8" t="inlineStr"/>
       <c r="H32" s="8" t="inlineStr"/>
       <c r="I32" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -49258,7 +49642,7 @@
       <c r="G33" s="8" t="inlineStr"/>
       <c r="H33" s="8" t="inlineStr"/>
       <c r="I33" s="8" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -49272,14 +49656,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -49478,7 +49862,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -50471,13 +50855,13 @@
         <v>1</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H32" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -50501,20 +50885,20 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F33" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H33" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
@@ -50831,7 +51215,7 @@
       <c r="G42" s="8" t="inlineStr"/>
       <c r="H42" s="8" t="inlineStr"/>
       <c r="I42" s="8" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43">
@@ -50886,7 +51270,7 @@
       <c r="C45" s="8" t="inlineStr"/>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr"/>
@@ -50894,24 +51278,45 @@
       <c r="G45" s="8" t="inlineStr"/>
       <c r="H45" s="8" t="inlineStr"/>
       <c r="I45" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr"/>
       <c r="C46" s="8" t="inlineStr"/>
-      <c r="D46" s="8" t="inlineStr"/>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Química</t>
+        </is>
+      </c>
       <c r="E46" s="8" t="inlineStr"/>
       <c r="F46" s="8" t="inlineStr"/>
       <c r="G46" s="8" t="inlineStr"/>
       <c r="H46" s="8" t="inlineStr"/>
       <c r="I46" s="8" t="n">
-        <v>93</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr"/>
+      <c r="C47" s="8" t="inlineStr"/>
+      <c r="D47" s="8" t="inlineStr"/>
+      <c r="E47" s="8" t="inlineStr"/>
+      <c r="F47" s="8" t="inlineStr"/>
+      <c r="G47" s="8" t="inlineStr"/>
+      <c r="H47" s="8" t="inlineStr"/>
+      <c r="I47" s="8" t="n">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -50925,14 +51330,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -51131,7 +51536,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -52198,13 +52603,13 @@
         <v>3</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H34" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -52228,20 +52633,20 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F35" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H35" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
@@ -52743,7 +53148,7 @@
       <c r="G49" s="8" t="inlineStr"/>
       <c r="H49" s="8" t="inlineStr"/>
       <c r="I49" s="8" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="50">
@@ -52798,7 +53203,7 @@
       <c r="C52" s="8" t="inlineStr"/>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr"/>
@@ -52806,24 +53211,45 @@
       <c r="G52" s="8" t="inlineStr"/>
       <c r="H52" s="8" t="inlineStr"/>
       <c r="I52" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr"/>
       <c r="C53" s="8" t="inlineStr"/>
-      <c r="D53" s="8" t="inlineStr"/>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Química</t>
+        </is>
+      </c>
       <c r="E53" s="8" t="inlineStr"/>
       <c r="F53" s="8" t="inlineStr"/>
       <c r="G53" s="8" t="inlineStr"/>
       <c r="H53" s="8" t="inlineStr"/>
       <c r="I53" s="8" t="n">
-        <v>113</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr"/>
+      <c r="C54" s="8" t="inlineStr"/>
+      <c r="D54" s="8" t="inlineStr"/>
+      <c r="E54" s="8" t="inlineStr"/>
+      <c r="F54" s="8" t="inlineStr"/>
+      <c r="G54" s="8" t="inlineStr"/>
+      <c r="H54" s="8" t="inlineStr"/>
+      <c r="I54" s="8" t="n">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -52837,7 +53263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -53043,7 +53469,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -54443,13 +54869,13 @@
         <v>2</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H43" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I43" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -54473,20 +54899,20 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H44" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
@@ -55028,7 +55454,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F59" s="5" t="n">
@@ -55358,7 +55784,7 @@
       <c r="G68" s="8" t="inlineStr"/>
       <c r="H68" s="8" t="inlineStr"/>
       <c r="I68" s="8" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69">
@@ -55413,7 +55839,7 @@
       <c r="C71" s="8" t="inlineStr"/>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr"/>
@@ -55421,7 +55847,7 @@
       <c r="G71" s="8" t="inlineStr"/>
       <c r="H71" s="8" t="inlineStr"/>
       <c r="I71" s="8" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72">
@@ -55434,7 +55860,7 @@
       <c r="C72" s="8" t="inlineStr"/>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr"/>
@@ -55442,7 +55868,7 @@
       <c r="G72" s="8" t="inlineStr"/>
       <c r="H72" s="8" t="inlineStr"/>
       <c r="I72" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
@@ -55455,7 +55881,7 @@
       <c r="C73" s="8" t="inlineStr"/>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr"/>
@@ -55463,24 +55889,45 @@
       <c r="G73" s="8" t="inlineStr"/>
       <c r="H73" s="8" t="inlineStr"/>
       <c r="I73" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr"/>
       <c r="C74" s="8" t="inlineStr"/>
-      <c r="D74" s="8" t="inlineStr"/>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E74" s="8" t="inlineStr"/>
       <c r="F74" s="8" t="inlineStr"/>
       <c r="G74" s="8" t="inlineStr"/>
       <c r="H74" s="8" t="inlineStr"/>
       <c r="I74" s="8" t="n">
-        <v>159</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr"/>
+      <c r="C75" s="8" t="inlineStr"/>
+      <c r="D75" s="8" t="inlineStr"/>
+      <c r="E75" s="8" t="inlineStr"/>
+      <c r="F75" s="8" t="inlineStr"/>
+      <c r="G75" s="8" t="inlineStr"/>
+      <c r="H75" s="8" t="inlineStr"/>
+      <c r="I75" s="8" t="n">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -55494,7 +55941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -55700,7 +56147,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -57359,13 +57806,13 @@
         <v>3</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H50" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -57389,20 +57836,20 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F51" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H51" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I51" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -57944,7 +58391,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F66" s="3" t="n">
@@ -58459,7 +58906,7 @@
       <c r="G80" s="8" t="inlineStr"/>
       <c r="H80" s="8" t="inlineStr"/>
       <c r="I80" s="8" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="81">
@@ -58514,7 +58961,7 @@
       <c r="C83" s="8" t="inlineStr"/>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr"/>
@@ -58522,7 +58969,7 @@
       <c r="G83" s="8" t="inlineStr"/>
       <c r="H83" s="8" t="inlineStr"/>
       <c r="I83" s="8" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="84">
@@ -58535,7 +58982,7 @@
       <c r="C84" s="8" t="inlineStr"/>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr"/>
@@ -58543,7 +58990,7 @@
       <c r="G84" s="8" t="inlineStr"/>
       <c r="H84" s="8" t="inlineStr"/>
       <c r="I84" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85">
@@ -58556,7 +59003,7 @@
       <c r="C85" s="8" t="inlineStr"/>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr"/>
@@ -58564,24 +59011,45 @@
       <c r="G85" s="8" t="inlineStr"/>
       <c r="H85" s="8" t="inlineStr"/>
       <c r="I85" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr"/>
       <c r="C86" s="8" t="inlineStr"/>
-      <c r="D86" s="8" t="inlineStr"/>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E86" s="8" t="inlineStr"/>
       <c r="F86" s="8" t="inlineStr"/>
       <c r="G86" s="8" t="inlineStr"/>
       <c r="H86" s="8" t="inlineStr"/>
       <c r="I86" s="8" t="n">
-        <v>188</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr"/>
+      <c r="C87" s="8" t="inlineStr"/>
+      <c r="D87" s="8" t="inlineStr"/>
+      <c r="E87" s="8" t="inlineStr"/>
+      <c r="F87" s="8" t="inlineStr"/>
+      <c r="G87" s="8" t="inlineStr"/>
+      <c r="H87" s="8" t="inlineStr"/>
+      <c r="I87" s="8" t="n">
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -58595,7 +59063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -58801,7 +59269,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -60429,7 +60897,7 @@
         <v>1</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -60719,13 +61187,13 @@
         <v>2</v>
       </c>
       <c r="G57" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H57" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I57" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -60749,20 +61217,20 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F58" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H58" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -61304,7 +61772,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F73" s="5" t="n">
@@ -61859,7 +62327,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="F88" s="3" t="n">
@@ -61893,7 +62361,7 @@
       <c r="G89" s="8" t="inlineStr"/>
       <c r="H89" s="8" t="inlineStr"/>
       <c r="I89" s="8" t="n">
-        <v>159</v>
+        <v>165</v>
       </c>
     </row>
     <row r="90">
@@ -61948,7 +62416,7 @@
       <c r="C92" s="8" t="inlineStr"/>
       <c r="D92" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Química</t>
+          <t>Laboratorio de Biología</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr"/>
@@ -61956,7 +62424,7 @@
       <c r="G92" s="8" t="inlineStr"/>
       <c r="H92" s="8" t="inlineStr"/>
       <c r="I92" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93">
@@ -61969,7 +62437,7 @@
       <c r="C93" s="8" t="inlineStr"/>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Computadoras</t>
+          <t>Laboratorio de Química</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr"/>
@@ -61977,7 +62445,7 @@
       <c r="G93" s="8" t="inlineStr"/>
       <c r="H93" s="8" t="inlineStr"/>
       <c r="I93" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">
@@ -61990,7 +62458,7 @@
       <c r="C94" s="8" t="inlineStr"/>
       <c r="D94" s="8" t="inlineStr">
         <is>
-          <t>Laboratorio de Física</t>
+          <t>Laboratorio de Computadoras</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr"/>
@@ -61998,24 +62466,45 @@
       <c r="G94" s="8" t="inlineStr"/>
       <c r="H94" s="8" t="inlineStr"/>
       <c r="I94" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr"/>
       <c r="C95" s="8" t="inlineStr"/>
-      <c r="D95" s="8" t="inlineStr"/>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Laboratorio de Física</t>
+        </is>
+      </c>
       <c r="E95" s="8" t="inlineStr"/>
       <c r="F95" s="8" t="inlineStr"/>
       <c r="G95" s="8" t="inlineStr"/>
       <c r="H95" s="8" t="inlineStr"/>
       <c r="I95" s="8" t="n">
-        <v>207</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr"/>
+      <c r="C96" s="8" t="inlineStr"/>
+      <c r="D96" s="8" t="inlineStr"/>
+      <c r="E96" s="8" t="inlineStr"/>
+      <c r="F96" s="8" t="inlineStr"/>
+      <c r="G96" s="8" t="inlineStr"/>
+      <c r="H96" s="8" t="inlineStr"/>
+      <c r="I96" s="8" t="n">
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>